<commit_message>
fix: reconcile provider TCO and isolate Excel cleanup failures
</commit_message>
<xml_diff>
--- a/skill-updates/2026-10-07/cloud-estimation-suite/examples/synthetic-cloud-estimate.xlsx
+++ b/skill-updates/2026-10-07/cloud-estimation-suite/examples/synthetic-cloud-estimate.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\skills\.worktrees\cloud-estimation-suite\skill-updates\2026-10-07\cloud-estimation-suite\examples\estimate-recalc-or_be79c\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\skills\.worktrees\cloud-estimation-suite\skill-updates\2026-10-07\cloud-estimation-suite\examples\estimate-recalc-p2vaafl1\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{a2896b27-184a-5fb0-8ec1-ebdfa757b35a}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ebda0527-cf2b-55cc-9c36-f211b8654afa}"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1040" uniqueCount="467">
   <si>
     <t>Lisez-moi</t>
   </si>
@@ -164,7 +164,7 @@
     <t>schedule.foundation_available</t>
   </si>
   <si>
-    <t>Period 1; role capacity 6 JH; dependency TASK-01 before TASK-02/09/10.</t>
+    <t>Period 1; collective capacity across Foundation roles, not per-role capacity. Owner: delivery lead. Dependency TASK-01 before TASK-02/09/10; individual role availability remains unverified.</t>
   </si>
   <si>
     <t>schedule.foundation_overload</t>
@@ -395,6 +395,12 @@
     <t>Explicit synthetic absence, not an unknown represented as zero.</t>
   </si>
   <si>
+    <t>comparison_scenario</t>
+  </si>
+  <si>
+    <t>Same reference scenario for all provider TCOs; independent of scenario_global, task overrides still apply.</t>
+  </si>
+  <si>
     <t>tco.ProviderA.Standard</t>
   </si>
   <si>
@@ -404,6 +410,18 @@
     <t>Dynamic selected Build plus 36 months of human Run, Provider A Standard cloud and non-cloud OPEX; alternatives never added.</t>
   </si>
   <si>
+    <t>tco.ProviderB.Standard</t>
+  </si>
+  <si>
+    <t>Dynamic same-perimeter Provider B comparison; Build, human Run, cloud and horizon remain separate in Scenarios.</t>
+  </si>
+  <si>
+    <t>tco.ProviderC.Standard</t>
+  </si>
+  <si>
+    <t>Dynamic same-perimeter Provider C comparison; alternatives never added.</t>
+  </si>
+  <si>
     <t>region_eligibility</t>
   </si>
   <si>
@@ -1109,6 +1127,24 @@
     <t>Uses high JH.</t>
   </si>
   <si>
+    <t>Comparaison fournisseurs - scenario de reference et horizon dans Hypotheses</t>
+  </si>
+  <si>
+    <t>Build (JH)</t>
+  </si>
+  <si>
+    <t>Run humain (JH/mois)</t>
+  </si>
+  <si>
+    <t>Cloud (EUR/mois)</t>
+  </si>
+  <si>
+    <t>Horizon (annees)</t>
+  </si>
+  <si>
+    <t>TCO (EUR)</t>
+  </si>
+  <si>
     <t>Phasage</t>
   </si>
   <si>
@@ -1298,7 +1334,7 @@
     <t>Move dependent Foundation work into another period before approval</t>
   </si>
   <si>
-    <t>Dynamic schedule.foundation_overload; capacity must be confirmed with role owner; subsequent periods cannot start before prerequisites. No approved calendar until overload is resolved.</t>
+    <t>Dynamic schedule.foundation_overload compares all Foundation Build with collective capacity, not a per-role budget. Delivery lead must confirm collective and individual role availability; subsequent periods cannot start before prerequisites. No approved calendar until overload is resolved.</t>
   </si>
   <si>
     <t>Sources</t>
@@ -1494,7 +1530,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1531,6 +1567,10 @@
     <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1601,51 +1641,67 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{2930ebf9-ed2a-5242-98b2-f548a6ab505a}" name="Arbitrages" displayName="Arbitrages" ref="A4:F9">
-  <autoFilter ref="A4:F9" xr:uid="{033658ed-4eec-5bc5-a115-38a32b766bba}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{c9c11c68-254a-5f28-aebf-20fe2601388a}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{fd20b698-64fe-551e-9b3c-e763d585e3ba}" name="Question"/>
-    <tableColumn id="3" xr3:uid="{2140a8fd-2180-5873-978d-375bad62986a}" name="Option"/>
-    <tableColumn id="4" xr3:uid="{c060f8c4-8d6a-5794-a1b1-0ddc8b69d10a}" name="Justification"/>
-    <tableColumn id="5" xr3:uid="{06082359-4097-5e1e-8198-0b6482f8c94a}" name="Statut"/>
-    <tableColumn id="6" xr3:uid="{d0a02626-4d6f-5c6c-8306-2ca6244508ea}" name="Source"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{cd4bbbae-a536-5bc4-acf0-7f289a4ea78a}" name="Risques" displayName="Risques" ref="A4:G8">
+  <autoFilter ref="A4:G8" xr:uid="{fcd4b4d2-5760-5384-9378-36325fb0bb0a}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{51e913c0-dca8-5f4a-9bb9-9e07078c91ea}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{0341ea9f-3146-5217-9034-f1c3fc3fd33a}" name="Risque"/>
+    <tableColumn id="3" xr3:uid="{6e489b8d-914a-590d-9a12-3817573b2cda}" name="Impact"/>
+    <tableColumn id="4" xr3:uid="{3a1e761d-d1e6-574d-9ed1-366aa80d590a}" name="Probabilite"/>
+    <tableColumn id="5" xr3:uid="{f8c5f345-5e61-539c-b4de-f894bb0e0a4a}" name="Mitigation"/>
+    <tableColumn id="6" xr3:uid="{50015aed-e4f6-5631-a8d7-85011555253a}" name="Responsable"/>
+    <tableColumn id="7" xr3:uid="{dda09037-fa1f-50c6-9289-dfce7ca0bd7a}" name="Statut"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{a45a3f82-d26b-55a1-b9a1-2b86b6a14f4a}" name="Sources" displayName="Sources" ref="A4:F7">
-  <autoFilter ref="A4:F7" xr:uid="{cd4bbbae-a536-5bc4-acf0-7f289a4ea78a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{1e90b6c6-2b17-5eff-a413-99c977e0a75a}" name="Arbitrages" displayName="Arbitrages" ref="A4:F9">
+  <autoFilter ref="A4:F9" xr:uid="{2bb47a34-ca22-5f0d-be8b-fb07986c2a6a}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{fcd4b4d2-5760-5384-9378-36325fb0bb0a}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{51e913c0-dca8-5f4a-9bb9-9e07078c91ea}" name="Titre"/>
-    <tableColumn id="3" xr3:uid="{0341ea9f-3146-5217-9034-f1c3fc3fd33a}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{6e489b8d-914a-590d-9a12-3817573b2cda}" name="Date"/>
-    <tableColumn id="5" xr3:uid="{3a1e761d-d1e6-574d-9ed1-366aa80d590a}" name="URL"/>
-    <tableColumn id="6" xr3:uid="{f8c5f345-5e61-539c-b4de-f894bb0e0a4a}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{50ba2783-800c-5507-a96b-ff15af196a3a}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{e63d4c41-e5ab-5d8b-8a78-04569dcededa}" name="Question"/>
+    <tableColumn id="3" xr3:uid="{3051fc14-4982-5cca-88e2-b60e736b1bfa}" name="Option"/>
+    <tableColumn id="4" xr3:uid="{20f46d42-3a4e-521e-abf2-2aae0bf0c91a}" name="Justification"/>
+    <tableColumn id="5" xr3:uid="{12839e61-f304-5141-b61a-51d54fdf1c7a}" name="Statut"/>
+    <tableColumn id="6" xr3:uid="{08e3c266-a13a-56ea-b410-8894895ac48a}" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{50015aed-e4f6-5631-a8d7-85011555253a}" name="Synthese" displayName="Synthese" ref="A4:D18">
-  <autoFilter ref="A4:D18" xr:uid="{dda09037-fa1f-50c6-9289-dfce7ca0bd7a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{89861eb7-7c63-52fd-b7bc-df26165ac67a}" name="Sources" displayName="Sources" ref="A4:F7">
+  <autoFilter ref="A4:F7" xr:uid="{69968ff6-2448-5986-a258-b6a2645d29ea}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{8c526499-7716-53af-b389-71adca89c33a}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{41f41fd3-8338-54a1-9e9b-eed66f803a8a}" name="Titre"/>
+    <tableColumn id="3" xr3:uid="{c453a05c-df26-5404-8632-6b40fc59bdea}" name="Type"/>
+    <tableColumn id="4" xr3:uid="{01de6852-72fd-558d-9214-9baa5ceb58da}" name="Date"/>
+    <tableColumn id="5" xr3:uid="{b4b60ff3-3cd1-5ab6-8ed5-f25f42af024a}" name="URL"/>
+    <tableColumn id="6" xr3:uid="{8d9c0c94-8824-51c1-9bce-b3b76d5db7ea}" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{1cdd1196-f545-52e5-ab48-b68c085421ea}" name="Synthese" displayName="Synthese" ref="A4:D18">
+  <autoFilter ref="A4:D18" xr:uid="{1a393a77-a4ef-5a69-9977-96635a3045fa}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{1e90b6c6-2b17-5eff-a413-99c977e0a75a}" name="Indicateur"/>
-    <tableColumn id="2" xr3:uid="{2bb47a34-ca22-5f0d-be8b-fb07986c2a6a}" name="Valeur"/>
-    <tableColumn id="3" xr3:uid="{50ba2783-800c-5507-a96b-ff15af196a3a}" name="Unite"/>
-    <tableColumn id="4" xr3:uid="{e63d4c41-e5ab-5d8b-8a78-04569dcededa}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{8fd71a24-d494-5f92-ae29-51a7d850dffa}" name="Indicateur"/>
+    <tableColumn id="2" xr3:uid="{4d41e4e9-7255-5bb9-b9df-a2a53cfce75a}" name="Valeur"/>
+    <tableColumn id="3" xr3:uid="{b2a75dd3-70b5-54b8-a132-f4a377fa570a}" name="Unite"/>
+    <tableColumn id="4" xr3:uid="{5d52df49-51c3-517f-b4b8-ceb0648488aa}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{aad93887-0d22-54b3-aecd-0bd71e83fd2a}" name="Hypotheses" displayName="Hypotheses" ref="A4:F46">
-  <autoFilter ref="A4:F46" xr:uid="{f503a2bc-b34e-550a-af3b-329339f9646a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{aad93887-0d22-54b3-aecd-0bd71e83fd2a}" name="Hypotheses" displayName="Hypotheses" ref="A4:F49">
+  <autoFilter ref="A4:F49" xr:uid="{f503a2bc-b34e-550a-af3b-329339f9646a}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9948146c-b1b7-50b3-b914-bb58fe15201a}" name="Hypothese"/>
     <tableColumn id="2" xr3:uid="{ef09338f-a6fd-5eae-ab17-1ee5a010ccfa}" name="Valeur"/>
@@ -1674,119 +1730,118 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{71c72121-6b34-592f-83cf-4e253a21a98a}" name="Architecture" displayName="Architecture" ref="A4:G6">
-  <autoFilter ref="A4:G6" xr:uid="{19121a22-bb51-59e5-8f7c-8eefa1edfc9a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4b2b67a0-ebe4-5e88-81a3-f9296e62f68a}" name="Architecture" displayName="Architecture" ref="A4:G6">
+  <autoFilter ref="A4:G6" xr:uid="{a843bed9-3533-54e4-b9df-7e769204124a}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{7d45de8b-4cd2-597d-87f1-fe4b8e3ab92a}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{401f235c-c4d3-5b1f-a85a-7af455ca672a}" name="Composant"/>
-    <tableColumn id="3" xr3:uid="{5df1a150-aa9b-52a4-87cd-9dae6aa3b32a}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{830ff998-77c8-517e-97ea-9361773d0dba}" name="Environnement"/>
-    <tableColumn id="5" xr3:uid="{92c4718d-0ed4-526e-bf94-0fc9f49f429a}" name="Fournisseur"/>
-    <tableColumn id="6" xr3:uid="{188942d6-baa4-520e-84d5-fac8d58875ca}" name="Decision"/>
-    <tableColumn id="7" xr3:uid="{7e067eba-da16-5f06-b593-a02933408d7a}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{2930d755-4929-5ead-890d-71c46bcde5ca}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{09e6e1f9-4c67-5ead-9fab-ef38bbe3e12a}" name="Composant"/>
+    <tableColumn id="3" xr3:uid="{2aa4be06-42dd-5921-9717-b8d6f316761a}" name="Type"/>
+    <tableColumn id="4" xr3:uid="{4177c298-77a6-51da-ba5c-148b8b82f1ca}" name="Environnement"/>
+    <tableColumn id="5" xr3:uid="{75196771-c594-5a35-b022-beef4f0de23a}" name="Fournisseur"/>
+    <tableColumn id="6" xr3:uid="{4f03187d-29c3-53a1-a5f7-466bffd52b0a}" name="Decision"/>
+    <tableColumn id="7" xr3:uid="{427836d2-cdfd-5e5e-b0f4-6123f6099aea}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{b7f4acee-7c87-5758-8753-1d06b18f44ca}" name="Taches" displayName="Taches" ref="A4:V14">
-  <autoFilter ref="A4:V14" xr:uid="{d3013e50-ef10-53dd-aed6-db74c418192a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0568ec0d-edd5-5e70-a25d-93073c260d0a}" name="Taches" displayName="Taches" ref="A4:V14">
+  <autoFilter ref="A4:V14" xr:uid="{ab5c54e6-12d9-5dac-b8a1-5903320f92ca}"/>
   <tableColumns count="22">
-    <tableColumn id="1" xr3:uid="{90ba6dc0-f861-5036-a267-1d5030eb682a}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{f56c8f09-61aa-5e9d-a7cb-19e3bb5be3da}" name="Lot"/>
-    <tableColumn id="3" xr3:uid="{dcef8d87-833d-572d-801c-704a88511fea}" name="Domaine"/>
-    <tableColumn id="4" xr3:uid="{1a70aba8-8390-5bfb-9b96-3ed6884c587a}" name="Tache"/>
-    <tableColumn id="5" xr3:uid="{7e0687be-9756-5fca-8c15-52d3b7db3d7a}" name="Livrable"/>
-    <tableColumn id="6" xr3:uid="{d19a4f0b-7083-5906-876b-081cb7b4073a}" name="Environnement"/>
-    <tableColumn id="7" xr3:uid="{dbe95fdd-5e22-5755-81ae-aac72aa1716a}" name="Role"/>
-    <tableColumn id="8" xr3:uid="{8917cddb-b932-5cf1-b599-8cd28c35b7ea}" name="Prerequis"/>
-    <tableColumn id="9" xr3:uid="{84504db3-3d4f-5ac5-b5b6-e7536aa7990a}" name="Dependances"/>
-    <tableColumn id="10" xr3:uid="{f3923dab-90c7-59ea-a686-e8386727e36a}" name="Critere d'acceptation"/>
-    <tableColumn id="11" xr3:uid="{9d6c779e-f880-55b9-9dbf-3a1228938dca}" name="Preuve attendue"/>
-    <tableColumn id="12" xr3:uid="{e63b9236-5c06-568a-8c32-e8b0bc3845da}" name="JH bas"/>
-    <tableColumn id="13" xr3:uid="{4f680658-df13-50b0-b529-1aa749392baa}" name="JH probable"/>
-    <tableColumn id="14" xr3:uid="{235cbb85-e01d-5154-989c-c6fa93ee786a}" name="JH haut"/>
-    <tableColumn id="15" xr3:uid="{9e39e5d5-89cd-5dea-b356-95b03d793d2a}" name="Scenario retenu"/>
-    <tableColumn id="16" xr3:uid="{9013c38a-d700-504c-8af7-db01b0e0c74a}" name="Scenario override"/>
-    <tableColumn id="17" xr3:uid="{0568ec0d-edd5-5e70-a25d-93073c260d0a}" name="JH retenu"/>
-    <tableColumn id="18" xr3:uid="{ab5c54e6-12d9-5dac-b8a1-5903320f92ca}" name="Nature"/>
-    <tableColumn id="19" xr3:uid="{8333a8e2-a5a5-5422-9d3d-a9d82123988a}" name="Couverture"/>
-    <tableColumn id="20" xr3:uid="{0b3cc4d1-5bcc-5d55-96e0-5736ba66d2ea}" name="Source"/>
-    <tableColumn id="21" xr3:uid="{d04ca565-6055-5889-9256-9a86cb0771fa}" name="Confiance"/>
-    <tableColumn id="22" xr3:uid="{66cf21f9-3f54-5a6d-a06f-856b02e133ba}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{8333a8e2-a5a5-5422-9d3d-a9d82123988a}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{0b3cc4d1-5bcc-5d55-96e0-5736ba66d2ea}" name="Lot"/>
+    <tableColumn id="3" xr3:uid="{d04ca565-6055-5889-9256-9a86cb0771fa}" name="Domaine"/>
+    <tableColumn id="4" xr3:uid="{66cf21f9-3f54-5a6d-a06f-856b02e133ba}" name="Tache"/>
+    <tableColumn id="5" xr3:uid="{fd5ea0e1-f66a-531d-8f5b-53bd8b5f944a}" name="Livrable"/>
+    <tableColumn id="6" xr3:uid="{784c2415-6e77-5e7e-96c4-09bef263fa6a}" name="Environnement"/>
+    <tableColumn id="7" xr3:uid="{b55476e7-caee-5375-8e22-9e92983fde5a}" name="Role"/>
+    <tableColumn id="8" xr3:uid="{2dab3fd7-3b82-55b2-a84b-5c7ce3453f0a}" name="Prerequis"/>
+    <tableColumn id="9" xr3:uid="{a5147cf5-8d22-58f5-ac60-7c7ba5ad6a8a}" name="Dependances"/>
+    <tableColumn id="10" xr3:uid="{aa5c09a5-bc66-561f-bc7c-0ef2f15a142a}" name="Critere d'acceptation"/>
+    <tableColumn id="11" xr3:uid="{284307cf-eac6-5bbf-8168-5cd3ade15d0a}" name="Preuve attendue"/>
+    <tableColumn id="12" xr3:uid="{5b910887-3827-5301-92c1-fb7318a78c4a}" name="JH bas"/>
+    <tableColumn id="13" xr3:uid="{e8092b37-5645-50fd-8c6a-7e9c8a70a0ba}" name="JH probable"/>
+    <tableColumn id="14" xr3:uid="{71c72121-6b34-592f-83cf-4e253a21a98a}" name="JH haut"/>
+    <tableColumn id="15" xr3:uid="{19121a22-bb51-59e5-8f7c-8eefa1edfc9a}" name="Scenario retenu"/>
+    <tableColumn id="16" xr3:uid="{7d45de8b-4cd2-597d-87f1-fe4b8e3ab92a}" name="Scenario override"/>
+    <tableColumn id="17" xr3:uid="{401f235c-c4d3-5b1f-a85a-7af455ca672a}" name="JH retenu"/>
+    <tableColumn id="18" xr3:uid="{5df1a150-aa9b-52a4-87cd-9dae6aa3b32a}" name="Nature"/>
+    <tableColumn id="19" xr3:uid="{830ff998-77c8-517e-97ea-9361773d0dba}" name="Couverture"/>
+    <tableColumn id="20" xr3:uid="{92c4718d-0ed4-526e-bf94-0fc9f49f429a}" name="Source"/>
+    <tableColumn id="21" xr3:uid="{188942d6-baa4-520e-84d5-fac8d58875ca}" name="Confiance"/>
+    <tableColumn id="22" xr3:uid="{7e067eba-da16-5f06-b593-a02933408d7a}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{c453a05c-df26-5404-8632-6b40fc59bdea}" name="CoutsCloud" displayName="CoutsCloud" ref="A4:P31">
-  <autoFilter ref="A4:P31" xr:uid="{01de6852-72fd-558d-9214-9baa5ceb58da}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{b7f4acee-7c87-5758-8753-1d06b18f44ca}" name="CoutsCloud" displayName="CoutsCloud" ref="A4:P31">
+  <autoFilter ref="A4:P31" xr:uid="{d3013e50-ef10-53dd-aed6-db74c418192a}"/>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{b4b60ff3-3cd1-5ab6-8ed5-f25f42af024a}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{8d9c0c94-8824-51c1-9bce-b3b76d5db7ea}" name="Fournisseur"/>
-    <tableColumn id="3" xr3:uid="{1cdd1196-f545-52e5-ab48-b68c085421ea}" name="Service"/>
-    <tableColumn id="4" xr3:uid="{1a393a77-a4ef-5a69-9977-96635a3045fa}" name="Environnement"/>
-    <tableColumn id="5" xr3:uid="{8fd71a24-d494-5f92-ae29-51a7d850dffa}" name="Scenario"/>
-    <tableColumn id="6" xr3:uid="{4d41e4e9-7255-5bb9-b9df-a2a53cfce75a}" name="Unite"/>
-    <tableColumn id="7" xr3:uid="{b2a75dd3-70b5-54b8-a132-f4a377fa570a}" name="Quantite"/>
-    <tableColumn id="8" xr3:uid="{5d52df49-51c3-517f-b4b8-ceb0648488aa}" name="Prix unitaire (EUR)"/>
-    <tableColumn id="9" xr3:uid="{12c0cb4d-569f-5108-818e-6f719f4fdcea}" name="Devise"/>
-    <tableColumn id="10" xr3:uid="{3a4aaff3-c659-5c1d-911d-165a52c45e2a}" name="Multiplicateur mensuel"/>
-    <tableColumn id="11" xr3:uid="{aa6cb732-7577-5b83-a6cf-130ff9df064a}" name="Cout mensuel (EUR)"/>
-    <tableColumn id="12" xr3:uid="{17d5dbf1-c329-5245-a03d-b56e7018a20a}" name="Cout annuel (EUR)"/>
-    <tableColumn id="13" xr3:uid="{67f4367c-4b6d-5d1a-81f9-ea8ead39433a}" name="Source"/>
-    <tableColumn id="14" xr3:uid="{50d47c37-00b7-5c68-af91-e08c8f4084ea}" name="Confiance"/>
-    <tableColumn id="15" xr3:uid="{d03b1108-473d-5b0b-b4b2-d4526ed4feba}" name="Notes"/>
-    <tableColumn id="16" xr3:uid="{9cf369e3-036d-5c1d-a389-8c4e364ee8ea}" name="Statut prix"/>
+    <tableColumn id="1" xr3:uid="{90ba6dc0-f861-5036-a267-1d5030eb682a}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{f56c8f09-61aa-5e9d-a7cb-19e3bb5be3da}" name="Fournisseur"/>
+    <tableColumn id="3" xr3:uid="{dcef8d87-833d-572d-801c-704a88511fea}" name="Service"/>
+    <tableColumn id="4" xr3:uid="{1a70aba8-8390-5bfb-9b96-3ed6884c587a}" name="Environnement"/>
+    <tableColumn id="5" xr3:uid="{7e0687be-9756-5fca-8c15-52d3b7db3d7a}" name="Scenario"/>
+    <tableColumn id="6" xr3:uid="{d19a4f0b-7083-5906-876b-081cb7b4073a}" name="Unite"/>
+    <tableColumn id="7" xr3:uid="{dbe95fdd-5e22-5755-81ae-aac72aa1716a}" name="Quantite"/>
+    <tableColumn id="8" xr3:uid="{8917cddb-b932-5cf1-b599-8cd28c35b7ea}" name="Prix unitaire (EUR)"/>
+    <tableColumn id="9" xr3:uid="{84504db3-3d4f-5ac5-b5b6-e7536aa7990a}" name="Devise"/>
+    <tableColumn id="10" xr3:uid="{f3923dab-90c7-59ea-a686-e8386727e36a}" name="Multiplicateur mensuel"/>
+    <tableColumn id="11" xr3:uid="{9d6c779e-f880-55b9-9dbf-3a1228938dca}" name="Cout mensuel (EUR)"/>
+    <tableColumn id="12" xr3:uid="{e63b9236-5c06-568a-8c32-e8b0bc3845da}" name="Cout annuel (EUR)"/>
+    <tableColumn id="13" xr3:uid="{4f680658-df13-50b0-b529-1aa749392baa}" name="Source"/>
+    <tableColumn id="14" xr3:uid="{235cbb85-e01d-5154-989c-c6fa93ee786a}" name="Confiance"/>
+    <tableColumn id="15" xr3:uid="{9e39e5d5-89cd-5dea-b356-95b03d793d2a}" name="Notes"/>
+    <tableColumn id="16" xr3:uid="{9013c38a-d700-504c-8af7-db01b0e0c74a}" name="Statut prix"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{3051fc14-4982-5cca-88e2-b60e736b1bfa}" name="Scenarios" displayName="Scenarios" ref="A4:F7">
-  <autoFilter ref="A4:F7" xr:uid="{20f46d42-3a4e-521e-abf2-2aae0bf0c91a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{12c0cb4d-569f-5108-818e-6f719f4fdcea}" name="Scenarios" displayName="Scenarios" ref="A4:F7">
+  <autoFilter ref="A4:F7" xr:uid="{3a4aaff3-c659-5c1d-911d-165a52c45e2a}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{12839e61-f304-5141-b61a-51d54fdf1c7a}" name="Scenario"/>
-    <tableColumn id="2" xr3:uid="{08e3c266-a13a-56ea-b410-8894895ac48a}" name="Description"/>
-    <tableColumn id="3" xr3:uid="{89861eb7-7c63-52fd-b7bc-df26165ac67a}" name="Rapprochement technique (non budgetaire)"/>
-    <tableColumn id="4" xr3:uid="{69968ff6-2448-5986-a258-b6a2645d29ea}" name="JH Build"/>
-    <tableColumn id="5" xr3:uid="{8c526499-7716-53af-b389-71adca89c33a}" name="JH Run/mois"/>
-    <tableColumn id="6" xr3:uid="{41f41fd3-8338-54a1-9e9b-eed66f803a8a}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{aa6cb732-7577-5b83-a6cf-130ff9df064a}" name="Scenario"/>
+    <tableColumn id="2" xr3:uid="{17d5dbf1-c329-5245-a03d-b56e7018a20a}" name="Description"/>
+    <tableColumn id="3" xr3:uid="{67f4367c-4b6d-5d1a-81f9-ea8ead39433a}" name="Rapprochement technique (non budgetaire)"/>
+    <tableColumn id="4" xr3:uid="{50d47c37-00b7-5c68-af91-e08c8f4084ea}" name="JH Build"/>
+    <tableColumn id="5" xr3:uid="{d03b1108-473d-5b0b-b4b2-d4526ed4feba}" name="JH Run/mois"/>
+    <tableColumn id="6" xr3:uid="{9cf369e3-036d-5c1d-a389-8c4e364ee8ea}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{fd5ea0e1-f66a-531d-8f5b-53bd8b5f944a}" name="Phasage" displayName="Phasage" ref="A4:G7">
-  <autoFilter ref="A4:G7" xr:uid="{784c2415-6e77-5e7e-96c4-09bef263fa6a}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{b55476e7-caee-5375-8e22-9e92983fde5a}" name="Phase"/>
-    <tableColumn id="2" xr3:uid="{2dab3fd7-3b82-55b2-a84b-5c7ce3453f0a}" name="Sequence"/>
-    <tableColumn id="3" xr3:uid="{a5147cf5-8d22-58f5-ac60-7c7ba5ad6a8a}" name="Jalon"/>
-    <tableColumn id="4" xr3:uid="{aa5c09a5-bc66-561f-bc7c-0ef2f15a142a}" name="Rapprochement technique (non budgetaire)"/>
-    <tableColumn id="5" xr3:uid="{284307cf-eac6-5bbf-8168-5cd3ade15d0a}" name="JH Build"/>
-    <tableColumn id="6" xr3:uid="{5b910887-3827-5301-92c1-fb7318a78c4a}" name="JH Run/mois"/>
-    <tableColumn id="7" xr3:uid="{e8092b37-5645-50fd-8c6a-7e9c8a70a0ba}" name="Notes"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{4f69d71a-ef47-5593-a27d-25207865c45a}" name="ComparaisonFournisseurs" displayName="ComparaisonFournisseurs" ref="A11:F14">
+  <autoFilter ref="A11:F14" xr:uid="{79159f42-91bc-5385-b3db-ac965ade843a}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{1fe21ff8-09f9-5fc5-8c43-55246d4138ea}" name="Fournisseur"/>
+    <tableColumn id="2" xr3:uid="{7da151ab-8bbe-5167-9ac8-591e571cdcea}" name="Build (JH)"/>
+    <tableColumn id="3" xr3:uid="{cb5cf7f8-0c10-583b-b4f2-1f09ba5bdfba}" name="Run humain (JH/mois)"/>
+    <tableColumn id="4" xr3:uid="{7eda38eb-4366-55ef-8f26-ed759cd8957a}" name="Cloud (EUR/mois)"/>
+    <tableColumn id="5" xr3:uid="{4d81f52c-e12d-5b71-90ac-7967b56f3faa}" name="Horizon (annees)"/>
+    <tableColumn id="6" xr3:uid="{3423e752-dbef-523b-bc74-d756fab16ffa}" name="TCO (EUR)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4b2b67a0-ebe4-5e88-81a3-f9296e62f68a}" name="Risques" displayName="Risques" ref="A4:G8">
-  <autoFilter ref="A4:G8" xr:uid="{a843bed9-3533-54e4-b9df-7e769204124a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2930ebf9-ed2a-5242-98b2-f548a6ab505a}" name="Phasage" displayName="Phasage" ref="A4:G7">
+  <autoFilter ref="A4:G7" xr:uid="{033658ed-4eec-5bc5-a115-38a32b766bba}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{2930d755-4929-5ead-890d-71c46bcde5ca}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{09e6e1f9-4c67-5ead-9fab-ef38bbe3e12a}" name="Risque"/>
-    <tableColumn id="3" xr3:uid="{2aa4be06-42dd-5921-9717-b8d6f316761a}" name="Impact"/>
-    <tableColumn id="4" xr3:uid="{4177c298-77a6-51da-ba5c-148b8b82f1ca}" name="Probabilite"/>
-    <tableColumn id="5" xr3:uid="{75196771-c594-5a35-b022-beef4f0de23a}" name="Mitigation"/>
-    <tableColumn id="6" xr3:uid="{4f03187d-29c3-53a1-a5f7-466bffd52b0a}" name="Responsable"/>
-    <tableColumn id="7" xr3:uid="{427836d2-cdfd-5e5e-b0f4-6123f6099aea}" name="Statut"/>
+    <tableColumn id="1" xr3:uid="{c9c11c68-254a-5f28-aebf-20fe2601388a}" name="Phase"/>
+    <tableColumn id="2" xr3:uid="{fd20b698-64fe-551e-9b3c-e763d585e3ba}" name="Sequence"/>
+    <tableColumn id="3" xr3:uid="{2140a8fd-2180-5873-978d-375bad62986a}" name="Jalon"/>
+    <tableColumn id="4" xr3:uid="{c060f8c4-8d6a-5794-a1b1-0ddc8b69d10a}" name="Rapprochement technique (non budgetaire)"/>
+    <tableColumn id="5" xr3:uid="{06082359-4097-5e1e-8198-0b6482f8c94a}" name="JH Build"/>
+    <tableColumn id="6" xr3:uid="{d0a02626-4d6f-5c6c-8306-2ca6244508ea}" name="JH Run/mois"/>
+    <tableColumn id="7" xr3:uid="{a45a3f82-d26b-55a1-b9a1-2b86b6a14f4a}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2166,26 +2221,26 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>390</v>
+        <v>402</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>391</v>
+        <v>403</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>392</v>
+        <v>404</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>393</v>
+        <v>405</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>394</v>
+        <v>406</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>18</v>
@@ -2196,16 +2251,16 @@
     </row>
     <row r="5" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>395</v>
+        <v>407</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>396</v>
+        <v>408</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>397</v>
+        <v>409</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>29</v>
@@ -2216,39 +2271,39 @@
     </row>
     <row r="6" spans="1:6" ht="285" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>398</v>
+        <v>410</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>400</v>
+        <v>412</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>401</v>
+        <v>413</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>402</v>
+        <v>414</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>403</v>
+        <v>415</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="285" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>405</v>
+        <v>417</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>406</v>
+        <v>418</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>407</v>
+        <v>419</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>25</v>
@@ -2256,39 +2311,39 @@
     </row>
     <row r="8" spans="1:6" ht="285" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>409</v>
+        <v>421</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>410</v>
+        <v>422</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>411</v>
+        <v>423</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>412</v>
+        <v>424</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>402</v>
+        <v>414</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="199.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="313.5" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>413</v>
+        <v>425</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>414</v>
+        <v>426</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>415</v>
+        <v>427</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>416</v>
+        <v>428</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>25</v>
@@ -2316,29 +2371,29 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>417</v>
+        <v>429</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>418</v>
+        <v>430</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>419</v>
+        <v>431</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>420</v>
+        <v>432</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>421</v>
+        <v>433</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>20</v>
@@ -2349,53 +2404,53 @@
         <v>25</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>422</v>
+        <v>434</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>423</v>
+        <v>435</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="4" t="s">
-        <v>424</v>
+        <v>436</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>425</v>
+        <v>437</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>426</v>
+        <v>438</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>423</v>
+        <v>435</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>427</v>
+        <v>439</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4" t="s">
-        <v>428</v>
+        <v>440</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="114" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>429</v>
+        <v>441</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>423</v>
+        <v>435</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E7" s="4"/>
       <c r="F7" s="4" t="s">
-        <v>431</v>
+        <v>443</v>
       </c>
     </row>
   </sheetData>
@@ -2420,17 +2475,17 @@
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>432</v>
+        <v>444</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>433</v>
+        <v>445</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>434</v>
+        <v>446</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>3</v>
@@ -2444,22 +2499,22 @@
     </row>
     <row r="5" spans="1:4" ht="99.75" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>435</v>
+        <v>447</v>
       </c>
       <c r="B5" s="10">
         <f>SUM(Taches[JH retenu])</f>
         <v>20</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>436</v>
+        <v>448</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>437</v>
+        <v>449</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="B6" s="10">
         <f>SUMIF(Taches[Nature],"Build",Taches[JH retenu])</f>
@@ -2469,12 +2524,12 @@
         <v>11</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>438</v>
+        <v>450</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>439</v>
+        <v>451</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIF(Taches[Nature],"Run",Taches[JH retenu])</f>
@@ -2484,12 +2539,12 @@
         <v>92</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>440</v>
+        <v>452</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>441</v>
+        <v>453</v>
       </c>
       <c r="B8" s="10">
         <f>SUMIF(Taches[Nature],"Build",Taches[JH retenu])*taux_journalier</f>
@@ -2499,12 +2554,12 @@
         <v>9</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>442</v>
+        <v>454</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>443</v>
+        <v>455</v>
       </c>
       <c r="B9" s="10">
         <f>SUMIF(Taches[Nature],"Run",Taches[JH retenu])*taux_journalier</f>
@@ -2514,12 +2569,12 @@
         <v>83</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>444</v>
+        <v>456</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>445</v>
+        <v>457</v>
       </c>
       <c r="B10" s="10">
         <f>SUMIFS(CoutsCloud[Cout mensuel (EUR)],CoutsCloud[Fournisseur],"Provider A",CoutsCloud[Scenario],"Economique")</f>
@@ -2529,12 +2584,12 @@
         <v>83</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>446</v>
+        <v>458</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>447</v>
+        <v>459</v>
       </c>
       <c r="B11" s="10">
         <f>SUMIFS(CoutsCloud[Cout mensuel (EUR)],CoutsCloud[Fournisseur],"Provider A",CoutsCloud[Scenario],"Standard")</f>
@@ -2544,12 +2599,12 @@
         <v>83</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>446</v>
+        <v>458</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>448</v>
+        <v>460</v>
       </c>
       <c r="B12" s="10">
         <f>SUMIFS(CoutsCloud[Cout mensuel (EUR)],CoutsCloud[Fournisseur],"Provider A",CoutsCloud[Scenario],"Resilient")</f>
@@ -2559,12 +2614,12 @@
         <v>83</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>446</v>
+        <v>458</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>449</v>
+        <v>461</v>
       </c>
       <c r="B13" s="10">
         <f>SUMIFS(CoutsCloud[Cout mensuel (EUR)],CoutsCloud[Fournisseur],"Provider B",CoutsCloud[Scenario],"Economique")</f>
@@ -2574,12 +2629,12 @@
         <v>83</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>446</v>
+        <v>458</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>450</v>
+        <v>462</v>
       </c>
       <c r="B14" s="10">
         <f>SUMIFS(CoutsCloud[Cout mensuel (EUR)],CoutsCloud[Fournisseur],"Provider B",CoutsCloud[Scenario],"Standard")</f>
@@ -2589,12 +2644,12 @@
         <v>83</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>446</v>
+        <v>458</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>451</v>
+        <v>463</v>
       </c>
       <c r="B15" s="10">
         <f>SUMIFS(CoutsCloud[Cout mensuel (EUR)],CoutsCloud[Fournisseur],"Provider B",CoutsCloud[Scenario],"Resilient")</f>
@@ -2604,12 +2659,12 @@
         <v>83</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>446</v>
+        <v>458</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>452</v>
+        <v>464</v>
       </c>
       <c r="B16" s="10">
         <f>SUMIFS(CoutsCloud[Cout mensuel (EUR)],CoutsCloud[Fournisseur],"Provider C",CoutsCloud[Scenario],"Economique")</f>
@@ -2619,12 +2674,12 @@
         <v>83</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>446</v>
+        <v>458</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>453</v>
+        <v>465</v>
       </c>
       <c r="B17" s="10">
         <f>SUMIFS(CoutsCloud[Cout mensuel (EUR)],CoutsCloud[Fournisseur],"Provider C",CoutsCloud[Scenario],"Standard")</f>
@@ -2634,12 +2689,12 @@
         <v>83</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>446</v>
+        <v>458</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>454</v>
+        <v>466</v>
       </c>
       <c r="B18" s="10">
         <f>SUMIFS(CoutsCloud[Cout mensuel (EUR)],CoutsCloud[Fournisseur],"Provider C",CoutsCloud[Scenario],"Resilient")</f>
@@ -2649,7 +2704,7 @@
         <v>83</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>446</v>
+        <v>458</v>
       </c>
     </row>
   </sheetData>
@@ -2666,7 +2721,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="6" width="16" customWidth="1"/>
@@ -2782,7 +2837,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="213.75" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>37</v>
       </c>
@@ -3450,76 +3505,78 @@
         <v>114</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="142.5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" ht="99.75" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="B42" s="12">
-        <f>'11_Synthese'!B8+('11_Synthese'!B9+'11_Synthese'!B11+B41)*mois_par_an*B40</f>
+      <c r="B42" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="142.5" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B43" s="12">
+        <f>'06_Scenarios'!F12</f>
         <v>41906</v>
       </c>
-      <c r="C42" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E42" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F42" s="5" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="85.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="5" t="s">
+      <c r="C43" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="D43" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F43" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="C43" s="5" t="s">
+    </row>
+    <row r="44" spans="1:6" ht="128.25" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="D43" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E43" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F43" s="5" t="s">
+      <c r="B44" s="12">
+        <f>'06_Scenarios'!F13</f>
+        <v>42446</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F44" s="5" t="s">
         <v>121</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="71.25" x14ac:dyDescent="0.25">
-      <c r="A44" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E44" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F44" s="5" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>126</v>
+        <v>122</v>
+      </c>
+      <c r="B45" s="12">
+        <f>'06_Scenarios'!F14</f>
+        <v>42986</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>29</v>
@@ -3528,27 +3585,87 @@
         <v>25</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="71.25" x14ac:dyDescent="0.25">
+      <c r="A47" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B47" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="C47" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F47" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="D46" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E46" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F46" s="5" t="s">
+    </row>
+    <row r="48" spans="1:6" ht="85.5" x14ac:dyDescent="0.25">
+      <c r="A48" s="5" t="s">
         <v>131</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="85.5" x14ac:dyDescent="0.25">
+      <c r="A49" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F49" s="5" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -3578,26 +3695,26 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>17</v>
@@ -3608,82 +3725,82 @@
     </row>
     <row r="5" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="D5" s="7">
         <v>1</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="D6" s="7">
         <v>1</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="D7" s="7">
         <v>2</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="142.5" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="D8" s="7">
         <v>1</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -3708,32 +3825,32 @@
   <sheetData>
     <row r="1" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>20</v>
@@ -3741,217 +3858,217 @@
     </row>
     <row r="5" spans="1:7" ht="199.5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="142.5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B18" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B24" s="9"/>
       <c r="C24" s="9" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B28" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -3983,77 +4100,77 @@
   <sheetData>
     <row r="1" spans="1:22" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" spans="1:22" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="T4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="U4" s="3" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="V4" s="3" t="s">
         <v>20</v>
@@ -4061,35 +4178,35 @@
     </row>
     <row r="5" spans="1:22" ht="99.75" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="L5" s="7">
         <v>2</v>
@@ -4110,54 +4227,54 @@
         <v>3</v>
       </c>
       <c r="R5" s="4" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="S5" s="4" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="T5" s="4" t="s">
         <v>25</v>
       </c>
       <c r="U5" s="4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="V5" s="4" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
     </row>
     <row r="6" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="L6" s="7">
         <v>1</v>
@@ -4173,61 +4290,61 @@
         <v>Resilient</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="Q6" s="11">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="T6" s="4" t="s">
         <v>25</v>
       </c>
       <c r="U6" s="4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="L7" s="7">
         <v>2</v>
@@ -4248,54 +4365,54 @@
         <v>3</v>
       </c>
       <c r="R7" s="4" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="S7" s="4" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="T7" s="4" t="s">
         <v>25</v>
       </c>
       <c r="U7" s="4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="V7" s="4" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
     </row>
     <row r="8" spans="1:22" ht="114" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="L8" s="7">
         <v>1</v>
@@ -4316,54 +4433,54 @@
         <v>2</v>
       </c>
       <c r="R8" s="4" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="S8" s="4" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="T8" s="4" t="s">
         <v>25</v>
       </c>
       <c r="U8" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="V8" s="4" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9" spans="1:22" ht="228" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="L9" s="7">
         <v>1</v>
@@ -4384,54 +4501,54 @@
         <v>2</v>
       </c>
       <c r="R9" s="4" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="S9" s="4" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="T9" s="4" t="s">
         <v>25</v>
       </c>
       <c r="U9" s="4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="V9" s="4" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="10" spans="1:22" ht="57" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="L10" s="7">
         <v>0.5</v>
@@ -4452,54 +4569,54 @@
         <v>1</v>
       </c>
       <c r="R10" s="4" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="S10" s="4" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="T10" s="4" t="s">
         <v>25</v>
       </c>
       <c r="U10" s="4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="V10" s="4" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11" spans="1:22" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="L11" s="7">
         <v>1</v>
@@ -4520,54 +4637,54 @@
         <v>2</v>
       </c>
       <c r="R11" s="4" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="S11" s="4" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="T11" s="4" t="s">
         <v>25</v>
       </c>
       <c r="U11" s="4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="V11" s="4" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
     <row r="12" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="L12" s="7">
         <v>0.5</v>
@@ -4588,54 +4705,54 @@
         <v>1</v>
       </c>
       <c r="R12" s="4" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="T12" s="4" t="s">
         <v>25</v>
       </c>
       <c r="U12" s="4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="V12" s="4" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
     <row r="13" spans="1:22" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="G13" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="I13" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="H13" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>207</v>
-      </c>
       <c r="J13" s="4" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="L13" s="7">
         <v>0.5</v>
@@ -4656,54 +4773,54 @@
         <v>1</v>
       </c>
       <c r="R13" s="4" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="S13" s="4" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="T13" s="4" t="s">
         <v>25</v>
       </c>
       <c r="U13" s="4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="V13" s="4" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
     <row r="14" spans="1:22" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="G14" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="I14" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="H14" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>207</v>
-      </c>
       <c r="J14" s="4" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="L14" s="7">
         <v>0.5</v>
@@ -4724,19 +4841,19 @@
         <v>1</v>
       </c>
       <c r="R14" s="4" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="S14" s="4" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="T14" s="4" t="s">
         <v>25</v>
       </c>
       <c r="U14" s="4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="V14" s="4" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>
@@ -4772,82 +4889,82 @@
   <sheetData>
     <row r="1" spans="1:16" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>17</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>20</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G5" s="7">
         <v>1</v>
@@ -4873,10 +4990,10 @@
         <v>25</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P5" s="4" t="s">
         <v>29</v>
@@ -4884,22 +5001,22 @@
     </row>
     <row r="6" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G6" s="7">
         <v>2</v>
@@ -4925,10 +5042,10 @@
         <v>25</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P6" s="4" t="s">
         <v>29</v>
@@ -4936,22 +5053,22 @@
     </row>
     <row r="7" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>313</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>314</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>308</v>
       </c>
       <c r="G7" s="7">
         <v>1</v>
@@ -4977,10 +5094,10 @@
         <v>25</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P7" s="4" t="s">
         <v>29</v>
@@ -4988,22 +5105,22 @@
     </row>
     <row r="8" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G8" s="7">
         <v>2</v>
@@ -5029,10 +5146,10 @@
         <v>25</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P8" s="4" t="s">
         <v>29</v>
@@ -5040,22 +5157,22 @@
     </row>
     <row r="9" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G9" s="7">
         <v>2</v>
@@ -5081,10 +5198,10 @@
         <v>25</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P9" s="4" t="s">
         <v>29</v>
@@ -5092,22 +5209,22 @@
     </row>
     <row r="10" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G10" s="7">
         <v>1</v>
@@ -5133,10 +5250,10 @@
         <v>25</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P10" s="4" t="s">
         <v>29</v>
@@ -5144,22 +5261,22 @@
     </row>
     <row r="11" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G11" s="7">
         <v>3</v>
@@ -5185,10 +5302,10 @@
         <v>25</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P11" s="4" t="s">
         <v>29</v>
@@ -5196,22 +5313,22 @@
     </row>
     <row r="12" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G12" s="7">
         <v>2</v>
@@ -5237,10 +5354,10 @@
         <v>25</v>
       </c>
       <c r="N12" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O12" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P12" s="4" t="s">
         <v>29</v>
@@ -5248,22 +5365,22 @@
     </row>
     <row r="13" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>320</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="F13" s="4" t="s">
         <v>314</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>308</v>
       </c>
       <c r="G13" s="7">
         <v>1</v>
@@ -5289,10 +5406,10 @@
         <v>25</v>
       </c>
       <c r="N13" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O13" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P13" s="4" t="s">
         <v>29</v>
@@ -5300,22 +5417,22 @@
     </row>
     <row r="14" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G14" s="7">
         <v>1</v>
@@ -5341,10 +5458,10 @@
         <v>25</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O14" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P14" s="4" t="s">
         <v>29</v>
@@ -5352,22 +5469,22 @@
     </row>
     <row r="15" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G15" s="7">
         <v>2</v>
@@ -5393,10 +5510,10 @@
         <v>25</v>
       </c>
       <c r="N15" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O15" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P15" s="4" t="s">
         <v>29</v>
@@ -5404,22 +5521,22 @@
     </row>
     <row r="16" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="C16" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>314</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>308</v>
       </c>
       <c r="G16" s="7">
         <v>1</v>
@@ -5445,10 +5562,10 @@
         <v>25</v>
       </c>
       <c r="N16" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O16" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P16" s="4" t="s">
         <v>29</v>
@@ -5456,22 +5573,22 @@
     </row>
     <row r="17" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G17" s="7">
         <v>2</v>
@@ -5497,10 +5614,10 @@
         <v>25</v>
       </c>
       <c r="N17" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O17" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P17" s="4" t="s">
         <v>29</v>
@@ -5508,22 +5625,22 @@
     </row>
     <row r="18" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G18" s="7">
         <v>2</v>
@@ -5549,10 +5666,10 @@
         <v>25</v>
       </c>
       <c r="N18" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O18" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P18" s="4" t="s">
         <v>29</v>
@@ -5560,22 +5677,22 @@
     </row>
     <row r="19" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G19" s="7">
         <v>1</v>
@@ -5601,10 +5718,10 @@
         <v>25</v>
       </c>
       <c r="N19" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P19" s="4" t="s">
         <v>29</v>
@@ -5612,22 +5729,22 @@
     </row>
     <row r="20" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>328</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>322</v>
-      </c>
       <c r="C20" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G20" s="7">
         <v>3</v>
@@ -5653,10 +5770,10 @@
         <v>25</v>
       </c>
       <c r="N20" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O20" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P20" s="4" t="s">
         <v>29</v>
@@ -5664,22 +5781,22 @@
     </row>
     <row r="21" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G21" s="7">
         <v>2</v>
@@ -5705,10 +5822,10 @@
         <v>25</v>
       </c>
       <c r="N21" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O21" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P21" s="4" t="s">
         <v>29</v>
@@ -5716,22 +5833,22 @@
     </row>
     <row r="22" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="C22" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>314</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>308</v>
       </c>
       <c r="G22" s="7">
         <v>1</v>
@@ -5757,10 +5874,10 @@
         <v>25</v>
       </c>
       <c r="N22" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O22" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P22" s="4" t="s">
         <v>29</v>
@@ -5768,22 +5885,22 @@
     </row>
     <row r="23" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G23" s="7">
         <v>1</v>
@@ -5809,10 +5926,10 @@
         <v>25</v>
       </c>
       <c r="N23" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O23" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P23" s="4" t="s">
         <v>29</v>
@@ -5820,22 +5937,22 @@
     </row>
     <row r="24" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G24" s="7">
         <v>2</v>
@@ -5861,10 +5978,10 @@
         <v>25</v>
       </c>
       <c r="N24" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O24" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P24" s="4" t="s">
         <v>29</v>
@@ -5872,22 +5989,22 @@
     </row>
     <row r="25" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="F25" s="4" t="s">
         <v>314</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>308</v>
       </c>
       <c r="G25" s="7">
         <v>1</v>
@@ -5913,10 +6030,10 @@
         <v>25</v>
       </c>
       <c r="N25" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O25" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P25" s="4" t="s">
         <v>29</v>
@@ -5924,22 +6041,22 @@
     </row>
     <row r="26" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G26" s="7">
         <v>2</v>
@@ -5965,10 +6082,10 @@
         <v>25</v>
       </c>
       <c r="N26" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O26" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P26" s="4" t="s">
         <v>29</v>
@@ -5976,22 +6093,22 @@
     </row>
     <row r="27" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G27" s="7">
         <v>2</v>
@@ -6017,10 +6134,10 @@
         <v>25</v>
       </c>
       <c r="N27" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O27" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P27" s="4" t="s">
         <v>29</v>
@@ -6028,22 +6145,22 @@
     </row>
     <row r="28" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G28" s="7">
         <v>1</v>
@@ -6069,10 +6186,10 @@
         <v>25</v>
       </c>
       <c r="N28" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O28" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P28" s="4" t="s">
         <v>29</v>
@@ -6080,22 +6197,22 @@
     </row>
     <row r="29" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>338</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>332</v>
-      </c>
       <c r="C29" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G29" s="7">
         <v>3</v>
@@ -6121,10 +6238,10 @@
         <v>25</v>
       </c>
       <c r="N29" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O29" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P29" s="4" t="s">
         <v>29</v>
@@ -6132,22 +6249,22 @@
     </row>
     <row r="30" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="G30" s="7">
         <v>2</v>
@@ -6173,10 +6290,10 @@
         <v>25</v>
       </c>
       <c r="N30" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O30" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P30" s="4" t="s">
         <v>29</v>
@@ -6184,22 +6301,22 @@
     </row>
     <row r="31" spans="1:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="C31" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="F31" s="4" t="s">
         <v>314</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>308</v>
       </c>
       <c r="G31" s="7">
         <v>1</v>
@@ -6225,10 +6342,10 @@
         <v>25</v>
       </c>
       <c r="N31" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="O31" s="4" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="P31" s="4" t="s">
         <v>29</v>
@@ -6248,7 +6365,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
@@ -6258,29 +6375,29 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>20</v>
@@ -6288,10 +6405,10 @@
     </row>
     <row r="5" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="C5" s="10">
         <f>SUM(Taches[JH bas])</f>
@@ -6306,7 +6423,7 @@
         <v>0.5</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
@@ -6314,7 +6431,7 @@
         <v>22</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="C6" s="10">
         <f>SUM(Taches[JH probable])</f>
@@ -6329,15 +6446,15 @@
         <v>1</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="C7" s="10">
         <f>SUM(Taches[JH haut])</f>
@@ -6352,14 +6469,115 @@
         <v>2</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>352</v>
+        <v>358</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>362</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>167</v>
+      </c>
+      <c r="B12" s="15">
+        <f>IF('01_Hypotheses'!B42="Economique",SUMIFS(Taches[JH bas],Taches[Nature],"Build",Taches[Scenario override],""),IF('01_Hypotheses'!B42="Standard",SUMIFS(Taches[JH probable],Taches[Nature],"Build",Taches[Scenario override],""),SUMIFS(Taches[JH haut],Taches[Nature],"Build",Taches[Scenario override],"")))+SUMIFS(Taches[JH bas],Taches[Nature],"Build",Taches[Scenario override],"Economique")+SUMIFS(Taches[JH probable],Taches[Nature],"Build",Taches[Scenario override],"Standard")+SUMIFS(Taches[JH haut],Taches[Nature],"Build",Taches[Scenario override],"Resilient")</f>
+        <v>19</v>
+      </c>
+      <c r="C12" s="15">
+        <f>IF('01_Hypotheses'!B42="Economique",SUMIFS(Taches[JH bas],Taches[Nature],"Run",Taches[Scenario override],""),IF('01_Hypotheses'!B42="Standard",SUMIFS(Taches[JH probable],Taches[Nature],"Run",Taches[Scenario override],""),SUMIFS(Taches[JH haut],Taches[Nature],"Run",Taches[Scenario override],"")))+SUMIFS(Taches[JH bas],Taches[Nature],"Run",Taches[Scenario override],"Economique")+SUMIFS(Taches[JH probable],Taches[Nature],"Run",Taches[Scenario override],"Standard")+SUMIFS(Taches[JH haut],Taches[Nature],"Run",Taches[Scenario override],"Resilient")</f>
+        <v>1</v>
+      </c>
+      <c r="D12" s="15">
+        <f>SUMIFS(CoutsCloud[Cout mensuel (EUR)],CoutsCloud[Fournisseur],A12,CoutsCloud[Scenario],'01_Hypotheses'!B42)</f>
+        <v>171</v>
+      </c>
+      <c r="E12" s="15">
+        <f>'01_Hypotheses'!B40</f>
+        <v>3</v>
+      </c>
+      <c r="F12" s="15">
+        <f>B12*taux_journalier+(C12*taux_journalier+D12+'01_Hypotheses'!B41)*mois_par_an*E12</f>
+        <v>41906</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>328</v>
+      </c>
+      <c r="B13" s="15">
+        <f>IF('01_Hypotheses'!B42="Economique",SUMIFS(Taches[JH bas],Taches[Nature],"Build",Taches[Scenario override],""),IF('01_Hypotheses'!B42="Standard",SUMIFS(Taches[JH probable],Taches[Nature],"Build",Taches[Scenario override],""),SUMIFS(Taches[JH haut],Taches[Nature],"Build",Taches[Scenario override],"")))+SUMIFS(Taches[JH bas],Taches[Nature],"Build",Taches[Scenario override],"Economique")+SUMIFS(Taches[JH probable],Taches[Nature],"Build",Taches[Scenario override],"Standard")+SUMIFS(Taches[JH haut],Taches[Nature],"Build",Taches[Scenario override],"Resilient")</f>
+        <v>19</v>
+      </c>
+      <c r="C13" s="15">
+        <f>IF('01_Hypotheses'!B42="Economique",SUMIFS(Taches[JH bas],Taches[Nature],"Run",Taches[Scenario override],""),IF('01_Hypotheses'!B42="Standard",SUMIFS(Taches[JH probable],Taches[Nature],"Run",Taches[Scenario override],""),SUMIFS(Taches[JH haut],Taches[Nature],"Run",Taches[Scenario override],"")))+SUMIFS(Taches[JH bas],Taches[Nature],"Run",Taches[Scenario override],"Economique")+SUMIFS(Taches[JH probable],Taches[Nature],"Run",Taches[Scenario override],"Standard")+SUMIFS(Taches[JH haut],Taches[Nature],"Run",Taches[Scenario override],"Resilient")</f>
+        <v>1</v>
+      </c>
+      <c r="D13" s="15">
+        <f>SUMIFS(CoutsCloud[Cout mensuel (EUR)],CoutsCloud[Fournisseur],A13,CoutsCloud[Scenario],'01_Hypotheses'!B42)</f>
+        <v>186</v>
+      </c>
+      <c r="E13" s="15">
+        <f>'01_Hypotheses'!B40</f>
+        <v>3</v>
+      </c>
+      <c r="F13" s="15">
+        <f>B13*taux_journalier+(C13*taux_journalier+D13+'01_Hypotheses'!B41)*mois_par_an*E13</f>
+        <v>42446</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>338</v>
+      </c>
+      <c r="B14" s="15">
+        <f>IF('01_Hypotheses'!B42="Economique",SUMIFS(Taches[JH bas],Taches[Nature],"Build",Taches[Scenario override],""),IF('01_Hypotheses'!B42="Standard",SUMIFS(Taches[JH probable],Taches[Nature],"Build",Taches[Scenario override],""),SUMIFS(Taches[JH haut],Taches[Nature],"Build",Taches[Scenario override],"")))+SUMIFS(Taches[JH bas],Taches[Nature],"Build",Taches[Scenario override],"Economique")+SUMIFS(Taches[JH probable],Taches[Nature],"Build",Taches[Scenario override],"Standard")+SUMIFS(Taches[JH haut],Taches[Nature],"Build",Taches[Scenario override],"Resilient")</f>
+        <v>19</v>
+      </c>
+      <c r="C14" s="15">
+        <f>IF('01_Hypotheses'!B42="Economique",SUMIFS(Taches[JH bas],Taches[Nature],"Run",Taches[Scenario override],""),IF('01_Hypotheses'!B42="Standard",SUMIFS(Taches[JH probable],Taches[Nature],"Run",Taches[Scenario override],""),SUMIFS(Taches[JH haut],Taches[Nature],"Run",Taches[Scenario override],"")))+SUMIFS(Taches[JH bas],Taches[Nature],"Run",Taches[Scenario override],"Economique")+SUMIFS(Taches[JH probable],Taches[Nature],"Run",Taches[Scenario override],"Standard")+SUMIFS(Taches[JH haut],Taches[Nature],"Run",Taches[Scenario override],"Resilient")</f>
+        <v>1</v>
+      </c>
+      <c r="D14" s="15">
+        <f>SUMIFS(CoutsCloud[Cout mensuel (EUR)],CoutsCloud[Fournisseur],A14,CoutsCloud[Scenario],'01_Hypotheses'!B42)</f>
+        <v>201</v>
+      </c>
+      <c r="E14" s="15">
+        <f>'01_Hypotheses'!B40</f>
+        <v>3</v>
+      </c>
+      <c r="F14" s="15">
+        <f>B14*taux_journalier+(C14*taux_journalier+D14+'01_Hypotheses'!B41)*mois_par_an*E14</f>
+        <v>42986</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="8" fitToHeight="0" orientation="landscape"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6379,32 +6597,32 @@
   <sheetData>
     <row r="1" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>353</v>
+        <v>365</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>354</v>
+        <v>366</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>355</v>
+        <v>367</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>357</v>
+        <v>369</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>20</v>
@@ -6412,13 +6630,13 @@
     </row>
     <row r="5" spans="1:7" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="B5" s="7">
         <v>1</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>358</v>
+        <v>370</v>
       </c>
       <c r="D5" s="10">
         <f>SUMIF(Taches[Lot],A5,Taches[JH retenu])</f>
@@ -6433,18 +6651,18 @@
         <v>0</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>359</v>
+        <v>371</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="B6" s="7">
         <v>2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="D6" s="10">
         <f>SUMIF(Taches[Lot],A6,Taches[JH retenu])</f>
@@ -6459,18 +6677,18 @@
         <v>0</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>361</v>
+        <v>373</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="B7" s="7">
         <v>3</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>362</v>
+        <v>374</v>
       </c>
       <c r="D7" s="10">
         <f>SUMIF(Taches[Lot],A7,Taches[JH retenu])</f>
@@ -6485,7 +6703,7 @@
         <v>1</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>363</v>
+        <v>375</v>
       </c>
     </row>
   </sheetData>
@@ -6510,32 +6728,32 @@
   <sheetData>
     <row r="1" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>364</v>
+        <v>376</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>365</v>
+        <v>377</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>366</v>
+        <v>378</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>367</v>
+        <v>379</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>368</v>
+        <v>380</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>370</v>
+        <v>382</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>18</v>
@@ -6543,94 +6761,94 @@
     </row>
     <row r="5" spans="1:7" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>372</v>
+        <v>384</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>377</v>
+        <v>389</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>378</v>
+        <v>390</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>379</v>
+        <v>391</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>381</v>
+        <v>393</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>382</v>
+        <v>394</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>383</v>
+        <v>395</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>384</v>
+        <v>396</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>385</v>
+        <v>397</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>386</v>
+        <v>398</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>387</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>388</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>389</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: verify cloud estimation skill delivery gates
</commit_message>
<xml_diff>
--- a/skill-updates/2026-10-07/cloud-estimation-suite/examples/synthetic-cloud-estimate.xlsx
+++ b/skill-updates/2026-10-07/cloud-estimation-suite/examples/synthetic-cloud-estimate.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\skills\.worktrees\cloud-estimation-suite\skill-updates\2026-10-07\cloud-estimation-suite\examples\estimate-recalc-p2vaafl1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\skills\.worktrees\cloud-estimation-suite\skill-updates\2026-10-07\cloud-estimation-suite\examples\estimate-recalc-6upzbrld\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{a2896b27-184a-5fb0-8ec1-ebdfa757b35a}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ebda0527-cf2b-55cc-9c36-f211b8654afa}"/>
@@ -3670,7 +3670,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" showErrorMessage="1" sqref="B5" xr:uid="{05521f1f-0f26-5f63-bcef-14c157ed415a}">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Scenario invalide" error="Choisir Economique, Standard ou Resilient." sqref="B5 B42" xr:uid="{05521f1f-0f26-5f63-bcef-14c157ed415a}">
       <formula1>"Economique,Standard,Resilient"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: preserve unknown finance and sanitize final estimation artifacts
</commit_message>
<xml_diff>
--- a/skill-updates/2026-10-07/cloud-estimation-suite/examples/synthetic-cloud-estimate.xlsx
+++ b/skill-updates/2026-10-07/cloud-estimation-suite/examples/synthetic-cloud-estimate.xlsx
@@ -4,13 +4,11 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\skills\.worktrees\cloud-estimation-suite\skill-updates\2026-10-07\cloud-estimation-suite\examples\estimate-recalc-6upzbrld\"/>
-    </mc:Choice>
+    <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{a2896b27-184a-5fb0-8ec1-ebdfa757b35a}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ebda0527-cf2b-55cc-9c36-f211b8654afa}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1ED6A53-15A4-49C5-AE55-4554CD7E4BC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{44752193-fdc5-5448-a654-697853f2665a}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Lisez-moi" sheetId="1" r:id="rId1"/>
@@ -48,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1040" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="470">
   <si>
     <t>Lisez-moi</t>
   </si>
@@ -626,7 +624,7 @@
     <t>JSON</t>
   </si>
   <si>
-    <t>{"edge_ids": ["FLOW-01"], "icon_provenance": [], "icon_sources": ["provider-neutral"], "node_ids": ["COMP-01", "COMP-02", "COMP-03", "COMP-04"], "output_hashes": {"png": "8c5879dd740af95745dc50167621d6b0cab18361906a09bf01ecfea18b0a0e45", "svg": "8a62826f1e0b0620086d42816296176f6bb8c192448511b9db76a620802468e6"}, "warnings": []}</t>
+    <t>{"edge_ids": ["FLOW-01"], "icon_provenance": [], "icon_sources": ["provider-neutral"], "node_ids": ["COMP-01", "COMP-02", "COMP-03", "COMP-04"], "output_hashes": {"png": "e0e2ec9c8c883554d77b86ce2bf5b328b61887fce74c656004457b9ae0aa4bf2", "svg": "24f1d21beb26437d7654dcddffaf415355f953121602a68fd44cdb12ef2c2150"}, "warnings": []}</t>
   </si>
   <si>
     <t>Taches_JH</t>
@@ -1449,6 +1447,15 @@
   </si>
   <si>
     <t>Cloud mensuel | Provider C | Resilient</t>
+  </si>
+  <si>
+    <t>Statut finance</t>
+  </si>
+  <si>
+    <t>Controle</t>
+  </si>
+  <si>
+    <t>Un taux inconnu bloque couts humains, TCO et approbation financiere, pas les capacites ou JH. Un taux renseigne ne vaut pas approbation.</t>
   </si>
 </sst>
 </file>
@@ -1578,10 +1585,10 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{b1c97f81-cc29-5329-addc-4ea2afb97f2a}">
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{c953488b-74be-50d7-8bc9-e3cef3f5885a}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
       <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
@@ -1602,8 +1609,8 @@
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
           <a:extLst>
-            <a:ext uri="{5a553d69-8e5b-51b5-aa41-5618b3bf3d8a}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96d79a94-4586-54a8-8198-b07ee6b9a60a}"/>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1630,218 +1637,218 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{31e5294d-3567-58ec-bcd1-a0135377dfca}" name="LisezMoi" displayName="LisezMoi" ref="A4:B9">
-  <autoFilter ref="A4:B9" xr:uid="{5aaffe1c-510f-5882-a924-2af90ea423ea}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="LisezMoi" displayName="LisezMoi" ref="A4:B9">
+  <autoFilter ref="A4:B9" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{640a6b42-bb53-5880-be40-ac65faae443a}" name="Cle"/>
-    <tableColumn id="2" xr3:uid="{8532d4c9-efd9-51c0-9579-cb7dc471835a}" name="Valeur"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Cle"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Valeur"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{cd4bbbae-a536-5bc4-acf0-7f289a4ea78a}" name="Risques" displayName="Risques" ref="A4:G8">
-  <autoFilter ref="A4:G8" xr:uid="{fcd4b4d2-5760-5384-9378-36325fb0bb0a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="Risques" displayName="Risques" ref="A4:G8">
+  <autoFilter ref="A4:G8" xr:uid="{00000000-0009-0000-0100-00000A000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{51e913c0-dca8-5f4a-9bb9-9e07078c91ea}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{0341ea9f-3146-5217-9034-f1c3fc3fd33a}" name="Risque"/>
-    <tableColumn id="3" xr3:uid="{6e489b8d-914a-590d-9a12-3817573b2cda}" name="Impact"/>
-    <tableColumn id="4" xr3:uid="{3a1e761d-d1e6-574d-9ed1-366aa80d590a}" name="Probabilite"/>
-    <tableColumn id="5" xr3:uid="{f8c5f345-5e61-539c-b4de-f894bb0e0a4a}" name="Mitigation"/>
-    <tableColumn id="6" xr3:uid="{50015aed-e4f6-5631-a8d7-85011555253a}" name="Responsable"/>
-    <tableColumn id="7" xr3:uid="{dda09037-fa1f-50c6-9289-dfce7ca0bd7a}" name="Statut"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="Risque"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0900-000003000000}" name="Impact"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0900-000004000000}" name="Probabilite"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0900-000005000000}" name="Mitigation"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0900-000006000000}" name="Responsable"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0900-000007000000}" name="Statut"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{1e90b6c6-2b17-5eff-a413-99c977e0a75a}" name="Arbitrages" displayName="Arbitrages" ref="A4:F9">
-  <autoFilter ref="A4:F9" xr:uid="{2bb47a34-ca22-5f0d-be8b-fb07986c2a6a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="Arbitrages" displayName="Arbitrages" ref="A4:F9">
+  <autoFilter ref="A4:F9" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{50ba2783-800c-5507-a96b-ff15af196a3a}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{e63d4c41-e5ab-5d8b-8a78-04569dcededa}" name="Question"/>
-    <tableColumn id="3" xr3:uid="{3051fc14-4982-5cca-88e2-b60e736b1bfa}" name="Option"/>
-    <tableColumn id="4" xr3:uid="{20f46d42-3a4e-521e-abf2-2aae0bf0c91a}" name="Justification"/>
-    <tableColumn id="5" xr3:uid="{12839e61-f304-5141-b61a-51d54fdf1c7a}" name="Statut"/>
-    <tableColumn id="6" xr3:uid="{08e3c266-a13a-56ea-b410-8894895ac48a}" name="Source"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Question"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="Option"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="Justification"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Statut"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0A00-000006000000}" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{89861eb7-7c63-52fd-b7bc-df26165ac67a}" name="Sources" displayName="Sources" ref="A4:F7">
-  <autoFilter ref="A4:F7" xr:uid="{69968ff6-2448-5986-a258-b6a2645d29ea}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{00000000-000C-0000-FFFF-FFFF0B000000}" name="Sources" displayName="Sources" ref="A4:F7">
+  <autoFilter ref="A4:F7" xr:uid="{00000000-0009-0000-0100-00000C000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{8c526499-7716-53af-b389-71adca89c33a}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{41f41fd3-8338-54a1-9e9b-eed66f803a8a}" name="Titre"/>
-    <tableColumn id="3" xr3:uid="{c453a05c-df26-5404-8632-6b40fc59bdea}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{01de6852-72fd-558d-9214-9baa5ceb58da}" name="Date"/>
-    <tableColumn id="5" xr3:uid="{b4b60ff3-3cd1-5ab6-8ed5-f25f42af024a}" name="URL"/>
-    <tableColumn id="6" xr3:uid="{8d9c0c94-8824-51c1-9bce-b3b76d5db7ea}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="Titre"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="Type"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="Date"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="URL"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{1cdd1196-f545-52e5-ab48-b68c085421ea}" name="Synthese" displayName="Synthese" ref="A4:D18">
-  <autoFilter ref="A4:D18" xr:uid="{1a393a77-a4ef-5a69-9977-96635a3045fa}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{00000000-000C-0000-FFFF-FFFF0C000000}" name="Synthese" displayName="Synthese" ref="A4:D19">
+  <autoFilter ref="A4:D19" xr:uid="{00000000-0009-0000-0100-00000D000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{8fd71a24-d494-5f92-ae29-51a7d850dffa}" name="Indicateur"/>
-    <tableColumn id="2" xr3:uid="{4d41e4e9-7255-5bb9-b9df-a2a53cfce75a}" name="Valeur"/>
-    <tableColumn id="3" xr3:uid="{b2a75dd3-70b5-54b8-a132-f4a377fa570a}" name="Unite"/>
-    <tableColumn id="4" xr3:uid="{5d52df49-51c3-517f-b4b8-ceb0648488aa}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0C00-000001000000}" name="Indicateur"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0C00-000002000000}" name="Valeur"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0C00-000003000000}" name="Unite"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0C00-000004000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{aad93887-0d22-54b3-aecd-0bd71e83fd2a}" name="Hypotheses" displayName="Hypotheses" ref="A4:F49">
-  <autoFilter ref="A4:F49" xr:uid="{f503a2bc-b34e-550a-af3b-329339f9646a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Hypotheses" displayName="Hypotheses" ref="A4:F49">
+  <autoFilter ref="A4:F49" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{9948146c-b1b7-50b3-b914-bb58fe15201a}" name="Hypothese"/>
-    <tableColumn id="2" xr3:uid="{ef09338f-a6fd-5eae-ab17-1ee5a010ccfa}" name="Valeur"/>
-    <tableColumn id="3" xr3:uid="{6e745675-1d20-522a-8991-f320fb9b596a}" name="Unite"/>
-    <tableColumn id="4" xr3:uid="{8ee9e152-805c-5090-9749-36abc42d926a}" name="Statut"/>
-    <tableColumn id="5" xr3:uid="{33a63bc0-8359-57e5-b280-e1aed4c4a3ca}" name="Source"/>
-    <tableColumn id="6" xr3:uid="{9ccee17c-5dd9-5b7f-bba7-66c1ed100efa}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Hypothese"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Valeur"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Unite"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Statut"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Source"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{f66f1d02-395e-54eb-9e60-0ed5719e151a}" name="Inventaire" displayName="Inventaire" ref="A4:F8">
-  <autoFilter ref="A4:F8" xr:uid="{d2d3b5c6-82d4-5356-b90f-7c58d26368ba}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Inventaire" displayName="Inventaire" ref="A4:F8">
+  <autoFilter ref="A4:F8" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{dab07832-1d81-58c1-b94b-811479073f5a}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{7a541b4b-3750-51d7-a93b-982ccadc09da}" name="Composant"/>
-    <tableColumn id="3" xr3:uid="{6d255b6a-38aa-5fe5-a3d3-2d01b64d9c3a}" name="Environnement"/>
-    <tableColumn id="4" xr3:uid="{82ae95d5-f4a8-53f6-8c1c-91fd5099db9a}" name="Quantite"/>
-    <tableColumn id="5" xr3:uid="{a584a42c-913b-5402-b032-a1ea3df2084a}" name="Unite"/>
-    <tableColumn id="6" xr3:uid="{0c784ac3-82c4-5d56-8500-645e99bd81ea}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Composant"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Environnement"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Quantite"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Unite"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4b2b67a0-ebe4-5e88-81a3-f9296e62f68a}" name="Architecture" displayName="Architecture" ref="A4:G6">
-  <autoFilter ref="A4:G6" xr:uid="{a843bed9-3533-54e4-b9df-7e769204124a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Architecture" displayName="Architecture" ref="A4:G6">
+  <autoFilter ref="A4:G6" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{2930d755-4929-5ead-890d-71c46bcde5ca}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{09e6e1f9-4c67-5ead-9fab-ef38bbe3e12a}" name="Composant"/>
-    <tableColumn id="3" xr3:uid="{2aa4be06-42dd-5921-9717-b8d6f316761a}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{4177c298-77a6-51da-ba5c-148b8b82f1ca}" name="Environnement"/>
-    <tableColumn id="5" xr3:uid="{75196771-c594-5a35-b022-beef4f0de23a}" name="Fournisseur"/>
-    <tableColumn id="6" xr3:uid="{4f03187d-29c3-53a1-a5f7-466bffd52b0a}" name="Decision"/>
-    <tableColumn id="7" xr3:uid="{427836d2-cdfd-5e5e-b0f4-6123f6099aea}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Composant"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Type"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Environnement"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Fournisseur"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Decision"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0568ec0d-edd5-5e70-a25d-93073c260d0a}" name="Taches" displayName="Taches" ref="A4:V14">
-  <autoFilter ref="A4:V14" xr:uid="{ab5c54e6-12d9-5dac-b8a1-5903320f92ca}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Taches" displayName="Taches" ref="A4:V14">
+  <autoFilter ref="A4:V14" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="22">
-    <tableColumn id="1" xr3:uid="{8333a8e2-a5a5-5422-9d3d-a9d82123988a}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{0b3cc4d1-5bcc-5d55-96e0-5736ba66d2ea}" name="Lot"/>
-    <tableColumn id="3" xr3:uid="{d04ca565-6055-5889-9256-9a86cb0771fa}" name="Domaine"/>
-    <tableColumn id="4" xr3:uid="{66cf21f9-3f54-5a6d-a06f-856b02e133ba}" name="Tache"/>
-    <tableColumn id="5" xr3:uid="{fd5ea0e1-f66a-531d-8f5b-53bd8b5f944a}" name="Livrable"/>
-    <tableColumn id="6" xr3:uid="{784c2415-6e77-5e7e-96c4-09bef263fa6a}" name="Environnement"/>
-    <tableColumn id="7" xr3:uid="{b55476e7-caee-5375-8e22-9e92983fde5a}" name="Role"/>
-    <tableColumn id="8" xr3:uid="{2dab3fd7-3b82-55b2-a84b-5c7ce3453f0a}" name="Prerequis"/>
-    <tableColumn id="9" xr3:uid="{a5147cf5-8d22-58f5-ac60-7c7ba5ad6a8a}" name="Dependances"/>
-    <tableColumn id="10" xr3:uid="{aa5c09a5-bc66-561f-bc7c-0ef2f15a142a}" name="Critere d'acceptation"/>
-    <tableColumn id="11" xr3:uid="{284307cf-eac6-5bbf-8168-5cd3ade15d0a}" name="Preuve attendue"/>
-    <tableColumn id="12" xr3:uid="{5b910887-3827-5301-92c1-fb7318a78c4a}" name="JH bas"/>
-    <tableColumn id="13" xr3:uid="{e8092b37-5645-50fd-8c6a-7e9c8a70a0ba}" name="JH probable"/>
-    <tableColumn id="14" xr3:uid="{71c72121-6b34-592f-83cf-4e253a21a98a}" name="JH haut"/>
-    <tableColumn id="15" xr3:uid="{19121a22-bb51-59e5-8f7c-8eefa1edfc9a}" name="Scenario retenu"/>
-    <tableColumn id="16" xr3:uid="{7d45de8b-4cd2-597d-87f1-fe4b8e3ab92a}" name="Scenario override"/>
-    <tableColumn id="17" xr3:uid="{401f235c-c4d3-5b1f-a85a-7af455ca672a}" name="JH retenu"/>
-    <tableColumn id="18" xr3:uid="{5df1a150-aa9b-52a4-87cd-9dae6aa3b32a}" name="Nature"/>
-    <tableColumn id="19" xr3:uid="{830ff998-77c8-517e-97ea-9361773d0dba}" name="Couverture"/>
-    <tableColumn id="20" xr3:uid="{92c4718d-0ed4-526e-bf94-0fc9f49f429a}" name="Source"/>
-    <tableColumn id="21" xr3:uid="{188942d6-baa4-520e-84d5-fac8d58875ca}" name="Confiance"/>
-    <tableColumn id="22" xr3:uid="{7e067eba-da16-5f06-b593-a02933408d7a}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Lot"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Domaine"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Tache"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Livrable"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="Environnement"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Role"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="Prerequis"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="Dependances"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0400-00000A000000}" name="Critere d'acceptation"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0400-00000B000000}" name="Preuve attendue"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0400-00000C000000}" name="JH bas"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0400-00000D000000}" name="JH probable"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0400-00000E000000}" name="JH haut"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0400-00000F000000}" name="Scenario retenu"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0400-000010000000}" name="Scenario override"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0400-000011000000}" name="JH retenu"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0400-000012000000}" name="Nature"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0400-000013000000}" name="Couverture"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0400-000014000000}" name="Source"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0400-000015000000}" name="Confiance"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0400-000016000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{b7f4acee-7c87-5758-8753-1d06b18f44ca}" name="CoutsCloud" displayName="CoutsCloud" ref="A4:P31">
-  <autoFilter ref="A4:P31" xr:uid="{d3013e50-ef10-53dd-aed6-db74c418192a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="CoutsCloud" displayName="CoutsCloud" ref="A4:P31">
+  <autoFilter ref="A4:P31" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{90ba6dc0-f861-5036-a267-1d5030eb682a}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{f56c8f09-61aa-5e9d-a7cb-19e3bb5be3da}" name="Fournisseur"/>
-    <tableColumn id="3" xr3:uid="{dcef8d87-833d-572d-801c-704a88511fea}" name="Service"/>
-    <tableColumn id="4" xr3:uid="{1a70aba8-8390-5bfb-9b96-3ed6884c587a}" name="Environnement"/>
-    <tableColumn id="5" xr3:uid="{7e0687be-9756-5fca-8c15-52d3b7db3d7a}" name="Scenario"/>
-    <tableColumn id="6" xr3:uid="{d19a4f0b-7083-5906-876b-081cb7b4073a}" name="Unite"/>
-    <tableColumn id="7" xr3:uid="{dbe95fdd-5e22-5755-81ae-aac72aa1716a}" name="Quantite"/>
-    <tableColumn id="8" xr3:uid="{8917cddb-b932-5cf1-b599-8cd28c35b7ea}" name="Prix unitaire (EUR)"/>
-    <tableColumn id="9" xr3:uid="{84504db3-3d4f-5ac5-b5b6-e7536aa7990a}" name="Devise"/>
-    <tableColumn id="10" xr3:uid="{f3923dab-90c7-59ea-a686-e8386727e36a}" name="Multiplicateur mensuel"/>
-    <tableColumn id="11" xr3:uid="{9d6c779e-f880-55b9-9dbf-3a1228938dca}" name="Cout mensuel (EUR)"/>
-    <tableColumn id="12" xr3:uid="{e63b9236-5c06-568a-8c32-e8b0bc3845da}" name="Cout annuel (EUR)"/>
-    <tableColumn id="13" xr3:uid="{4f680658-df13-50b0-b529-1aa749392baa}" name="Source"/>
-    <tableColumn id="14" xr3:uid="{235cbb85-e01d-5154-989c-c6fa93ee786a}" name="Confiance"/>
-    <tableColumn id="15" xr3:uid="{9e39e5d5-89cd-5dea-b356-95b03d793d2a}" name="Notes"/>
-    <tableColumn id="16" xr3:uid="{9013c38a-d700-504c-8af7-db01b0e0c74a}" name="Statut prix"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Fournisseur"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Service"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Environnement"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Scenario"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Unite"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="Quantite"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="Prix unitaire (EUR)"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="Devise"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" name="Multiplicateur mensuel"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0500-00000B000000}" name="Cout mensuel (EUR)"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0500-00000C000000}" name="Cout annuel (EUR)"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0500-00000D000000}" name="Source"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0500-00000E000000}" name="Confiance"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0500-00000F000000}" name="Notes"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0500-000010000000}" name="Statut prix"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{12c0cb4d-569f-5108-818e-6f719f4fdcea}" name="Scenarios" displayName="Scenarios" ref="A4:F7">
-  <autoFilter ref="A4:F7" xr:uid="{3a4aaff3-c659-5c1d-911d-165a52c45e2a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Scenarios" displayName="Scenarios" ref="A4:F7">
+  <autoFilter ref="A4:F7" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{aa6cb732-7577-5b83-a6cf-130ff9df064a}" name="Scenario"/>
-    <tableColumn id="2" xr3:uid="{17d5dbf1-c329-5245-a03d-b56e7018a20a}" name="Description"/>
-    <tableColumn id="3" xr3:uid="{67f4367c-4b6d-5d1a-81f9-ea8ead39433a}" name="Rapprochement technique (non budgetaire)"/>
-    <tableColumn id="4" xr3:uid="{50d47c37-00b7-5c68-af91-e08c8f4084ea}" name="JH Build"/>
-    <tableColumn id="5" xr3:uid="{d03b1108-473d-5b0b-b4b2-d4526ed4feba}" name="JH Run/mois"/>
-    <tableColumn id="6" xr3:uid="{9cf369e3-036d-5c1d-a389-8c4e364ee8ea}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="Scenario"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Description"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Rapprochement technique (non budgetaire)"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="JH Build"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="JH Run/mois"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{4f69d71a-ef47-5593-a27d-25207865c45a}" name="ComparaisonFournisseurs" displayName="ComparaisonFournisseurs" ref="A11:F14">
-  <autoFilter ref="A11:F14" xr:uid="{79159f42-91bc-5385-b3db-ac965ade843a}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="ComparaisonFournisseurs" displayName="ComparaisonFournisseurs" ref="A11:F14">
+  <autoFilter ref="A11:F14" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{1fe21ff8-09f9-5fc5-8c43-55246d4138ea}" name="Fournisseur"/>
-    <tableColumn id="2" xr3:uid="{7da151ab-8bbe-5167-9ac8-591e571cdcea}" name="Build (JH)"/>
-    <tableColumn id="3" xr3:uid="{cb5cf7f8-0c10-583b-b4f2-1f09ba5bdfba}" name="Run humain (JH/mois)"/>
-    <tableColumn id="4" xr3:uid="{7eda38eb-4366-55ef-8f26-ed759cd8957a}" name="Cloud (EUR/mois)"/>
-    <tableColumn id="5" xr3:uid="{4d81f52c-e12d-5b71-90ac-7967b56f3faa}" name="Horizon (annees)"/>
-    <tableColumn id="6" xr3:uid="{3423e752-dbef-523b-bc74-d756fab16ffa}" name="TCO (EUR)"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Fournisseur"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Build (JH)"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Run humain (JH/mois)"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Cloud (EUR/mois)"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="Horizon (annees)"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="TCO (EUR)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2930ebf9-ed2a-5242-98b2-f548a6ab505a}" name="Phasage" displayName="Phasage" ref="A4:G7">
-  <autoFilter ref="A4:G7" xr:uid="{033658ed-4eec-5bc5-a115-38a32b766bba}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Phasage" displayName="Phasage" ref="A4:G7">
+  <autoFilter ref="A4:G7" xr:uid="{00000000-0009-0000-0100-000009000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{c9c11c68-254a-5f28-aebf-20fe2601388a}" name="Phase"/>
-    <tableColumn id="2" xr3:uid="{fd20b698-64fe-551e-9b3c-e763d585e3ba}" name="Sequence"/>
-    <tableColumn id="3" xr3:uid="{2140a8fd-2180-5873-978d-375bad62986a}" name="Jalon"/>
-    <tableColumn id="4" xr3:uid="{c060f8c4-8d6a-5794-a1b1-0ddc8b69d10a}" name="Rapprochement technique (non budgetaire)"/>
-    <tableColumn id="5" xr3:uid="{06082359-4097-5e1e-8198-0b6482f8c94a}" name="JH Build"/>
-    <tableColumn id="6" xr3:uid="{d0a02626-4d6f-5c6c-8306-2ca6244508ea}" name="JH Run/mois"/>
-    <tableColumn id="7" xr3:uid="{a45a3f82-d26b-55a1-b9a1-2b86b6a14f4a}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="Phase"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="Sequence"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="Jalon"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="Rapprochement technique (non budgetaire)"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="JH Build"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="JH Run/mois"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2131,7 +2138,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9a997289-9c99-50f4-9a50-6ab01beabf4a}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2209,7 +2216,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{de4fa7d0-0a90-5461-8c8c-d40a600ecc8a}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2359,7 +2366,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49e0cb1f-89e5-5316-beaf-712b2c02ed5a}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2463,11 +2470,11 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{708f7b2c-c475-54bd-b4e0-a63ecedaefda}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="16" customWidth="1"/>
@@ -2547,7 +2554,7 @@
         <v>453</v>
       </c>
       <c r="B8" s="10">
-        <f>SUMIF(Taches[Nature],"Build",Taches[JH retenu])*taux_journalier</f>
+        <f>IF(taux_journalier="","",IF(taux_journalier="A chiffrer","",SUMIF(Taches[Nature],"Build",Taches[JH retenu])*taux_journalier))</f>
         <v>12350</v>
       </c>
       <c r="C8" s="4" t="s">
@@ -2562,7 +2569,7 @@
         <v>455</v>
       </c>
       <c r="B9" s="10">
-        <f>SUMIF(Taches[Nature],"Run",Taches[JH retenu])*taux_journalier</f>
+        <f>IF(taux_journalier="","",IF(taux_journalier="A chiffrer","",SUMIF(Taches[Nature],"Run",Taches[JH retenu])*taux_journalier))</f>
         <v>650</v>
       </c>
       <c r="C9" s="4" t="s">
@@ -2705,6 +2712,21 @@
       </c>
       <c r="D18" s="4" t="s">
         <v>458</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="142.5" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="B19" s="10" t="str">
+        <f>IF(taux_journalier="","Bloque - taux journalier A chiffrer",IF(taux_journalier="A chiffrer","Bloque - taux journalier A chiffrer","Taux journalier renseigne - approbation non acquise"))</f>
+        <v>Taux journalier renseigne - approbation non acquise</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>469</v>
       </c>
     </row>
   </sheetData>
@@ -2717,7 +2739,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2a9efe25-8ca8-52ca-bf8b-ecb71db732ba}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3670,7 +3692,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Scenario invalide" error="Choisir Economique, Standard ou Resilient." sqref="B5 B42" xr:uid="{05521f1f-0f26-5f63-bcef-14c157ed415a}">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Scenario invalide" error="Choisir Economique, Standard ou Resilient." sqref="B5 B42" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Economique,Standard,Resilient"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3683,7 +3705,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4e37a443-61cd-5c9e-ad20-5d2d1f7142aa}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3813,7 +3835,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ab7856c7-5124-5f82-b405-ce1ea86e5a3a}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -4082,7 +4104,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{621fe676-534f-5e80-adb8-a93dc91ed40a}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -4858,7 +4880,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Scenario invalide" error="Choisir un scenario de la liste." sqref="P5:P14" xr:uid="{ab391359-3fef-5489-a52d-a8c97afc5e5a}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Scenario invalide" error="Choisir un scenario de la liste." sqref="P5:P14" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"Economique,Standard,Resilient"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4871,7 +4893,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82958636-9a66-52aa-a9c4-16358b0f4d3a}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -6361,7 +6383,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17ab95de-9d0e-54f7-9289-8db01200976a}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -6518,7 +6540,7 @@
         <v>3</v>
       </c>
       <c r="F12" s="15">
-        <f>B12*taux_journalier+(C12*taux_journalier+D12+'01_Hypotheses'!B41)*mois_par_an*E12</f>
+        <f>IF(taux_journalier="","",IF(taux_journalier="A chiffrer","",B12*taux_journalier+(C12*taux_journalier+D12+'01_Hypotheses'!B41)*mois_par_an*E12))</f>
         <v>41906</v>
       </c>
     </row>
@@ -6543,7 +6565,7 @@
         <v>3</v>
       </c>
       <c r="F13" s="15">
-        <f>B13*taux_journalier+(C13*taux_journalier+D13+'01_Hypotheses'!B41)*mois_par_an*E13</f>
+        <f>IF(taux_journalier="","",IF(taux_journalier="A chiffrer","",B13*taux_journalier+(C13*taux_journalier+D13+'01_Hypotheses'!B41)*mois_par_an*E13))</f>
         <v>42446</v>
       </c>
     </row>
@@ -6568,7 +6590,7 @@
         <v>3</v>
       </c>
       <c r="F14" s="15">
-        <f>B14*taux_journalier+(C14*taux_journalier+D14+'01_Hypotheses'!B41)*mois_par_an*E14</f>
+        <f>IF(taux_journalier="","",IF(taux_journalier="A chiffrer","",B14*taux_journalier+(C14*taux_journalier+D14+'01_Hypotheses'!B41)*mois_par_an*E14))</f>
         <v>42986</v>
       </c>
     </row>
@@ -6583,7 +6605,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26e74fb5-b4b7-5e46-8ff3-fc76284e7f4a}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -6716,7 +6738,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ba4d852-59f4-56f0-962f-74f93829f02a}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>

<commit_message>
fix: preserve raster separation and flow identity in diagrams
</commit_message>
<xml_diff>
--- a/skill-updates/2026-10-07/cloud-estimation-suite/examples/synthetic-cloud-estimate.xlsx
+++ b/skill-updates/2026-10-07/cloud-estimation-suite/examples/synthetic-cloud-estimate.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E62B907-BC0A-4C6A-AEB4-5FDC78FF4234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{303E1A76-D4FA-47DD-A141-3CCA9B71CDD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -624,7 +624,7 @@
     <t>JSON</t>
   </si>
   <si>
-    <t>{"edge_ids": ["FLOW-01"], "icon_provenance": [], "icon_sources": ["provider-neutral"], "node_ids": ["COMP-01", "COMP-02", "COMP-03", "COMP-04"], "output_hashes": {"png": "29908a7330c509dfb1b8cf18fb12a5b675699b1297dc0adebe921f692e82afc6", "svg": "71725f3c9a4a48719f40374c8a9b7fbd49ef72762b53d572fab1b6a4e20184eb"}, "warnings": []}</t>
+    <t>{"edge_ids": ["FLOW-01"], "icon_provenance": [], "icon_sources": ["provider-neutral"], "node_ids": ["COMP-01", "COMP-02", "COMP-03", "COMP-04"], "output_hashes": {"png": "b974403dc6b60ce6ee2807f5d4d4c7c2f97f39c3f271e86d5c77631bec2a8012", "svg": "dc33f5574f3991d64fc15713506792ead06eec47d5dd3d9e4591835ca27e8042"}, "warnings": []}</t>
   </si>
   <si>
     <t>Taches_JH</t>
@@ -1604,7 +1604,7 @@
       <xdr:row>30</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="6477000" cy="9715500"/>
+    <xdr:ext cx="9829800" cy="14630400"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">

</xml_diff>

<commit_message>
fix: add Unicode font metadata and renderer support
</commit_message>
<xml_diff>
--- a/skill-updates/2026-10-07/cloud-estimation-suite/examples/synthetic-cloud-estimate.xlsx
+++ b/skill-updates/2026-10-07/cloud-estimation-suite/examples/synthetic-cloud-estimate.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7488CA5D-1A4C-426F-B786-856B7CA0C028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E62B907-BC0A-4C6A-AEB4-5FDC78FF4234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -624,7 +624,7 @@
     <t>JSON</t>
   </si>
   <si>
-    <t>{"edge_ids": ["FLOW-01"], "icon_provenance": [], "icon_sources": ["provider-neutral"], "node_ids": ["COMP-01", "COMP-02", "COMP-03", "COMP-04"], "output_hashes": {"png": "e0e2ec9c8c883554d77b86ce2bf5b328b61887fce74c656004457b9ae0aa4bf2", "svg": "24f1d21beb26437d7654dcddffaf415355f953121602a68fd44cdb12ef2c2150"}, "warnings": []}</t>
+    <t>{"edge_ids": ["FLOW-01"], "icon_provenance": [], "icon_sources": ["provider-neutral"], "node_ids": ["COMP-01", "COMP-02", "COMP-03", "COMP-04"], "output_hashes": {"png": "29908a7330c509dfb1b8cf18fb12a5b675699b1297dc0adebe921f692e82afc6", "svg": "71725f3c9a4a48719f40374c8a9b7fbd49ef72762b53d572fab1b6a4e20184eb"}, "warnings": []}</t>
   </si>
   <si>
     <t>Taches_JH</t>

</xml_diff>